<commit_message>
Fix rilievi C011/C007: aggiornati report-checklist, data.json e FILES/SIGNED
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#INFO99SASXX/INFO99_SAS/GLAB400/2.30/report-checklist.xlsx
+++ b/GATEWAY/A1#111#INFO99SASXX/INFO99_SAS/GLAB400/2.30/report-checklist.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="33720" yWindow="975" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni Compilazione" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prerequisiti" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestCases" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISTA VALORI" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="Istruzioni Compilazione" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Prerequisiti" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TestCases" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="LISTA VALORI" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TestCases'!$A$9:$W$190</definedName>
@@ -2600,7 +2600,7 @@
       </c>
       <c r="H10" s="36" t="inlineStr">
         <is>
-          <t>bca91958642e9381485555f996bfa4d7a88762d1e9f3ebfe6ec9783e1415303d</t>
+          <t>8b7d8a883260a8afb47d70cec6c307db</t>
         </is>
       </c>
       <c r="I10" s="60" t="inlineStr">
@@ -2615,12 +2615,32 @@
       </c>
       <c r="K10" s="62" t="n"/>
       <c r="L10" s="62" t="n"/>
-      <c r="M10" s="62" t="n"/>
-      <c r="N10" s="62" t="n"/>
+      <c r="M10" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="N10" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="O10" s="62" t="n"/>
-      <c r="P10" s="62" t="n"/>
-      <c r="Q10" s="62" t="n"/>
-      <c r="R10" s="62" t="n"/>
+      <c r="P10" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q10" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R10" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="S10" s="62" t="n"/>
       <c r="T10" s="62" t="inlineStr">
         <is>
@@ -2663,29 +2683,77 @@
 Al fine di rendere non valido il token è necessario non valorizzare nel JWT il campo "purpose_of_use".</t>
         </is>
       </c>
-      <c r="F11" s="60" t="n"/>
-      <c r="G11" s="60" t="n"/>
-      <c r="H11" s="60" t="n"/>
-      <c r="I11" s="61" t="n"/>
+      <c r="F11" s="60" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="G11" s="60" t="inlineStr">
+        <is>
+          <t>2026-03-03 09:01:58</t>
+        </is>
+      </c>
+      <c r="H11" s="60" t="inlineStr">
+        <is>
+          <t>14a167126aa14a042dcb7aec04a4f76a</t>
+        </is>
+      </c>
+      <c r="I11" s="61" t="inlineStr">
+        <is>
+          <t>UNKNOWN_WORKFLOW_ID</t>
+        </is>
+      </c>
       <c r="J11" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K11" s="62" t="inlineStr">
+        <is>
+          <t>Campo obbligatorio</t>
+        </is>
+      </c>
+      <c r="L11" s="62" t="n"/>
+      <c r="M11" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N11" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="O11" s="62" t="inlineStr">
+        <is>
+          <t>Il campo purpose_of_use non Ã¨ valorizzato</t>
+        </is>
+      </c>
+      <c r="P11" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q11" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R11" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="K11" s="62" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
-      <c r="L11" s="62" t="n"/>
-      <c r="M11" s="62" t="n"/>
-      <c r="N11" s="62" t="n"/>
-      <c r="O11" s="62" t="n"/>
-      <c r="P11" s="62" t="n"/>
-      <c r="Q11" s="62" t="n"/>
-      <c r="R11" s="62" t="n"/>
-      <c r="S11" s="62" t="n"/>
-      <c r="T11" s="62" t="n"/>
+      <c r="S11" s="62" t="inlineStr">
+        <is>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
+        </is>
+      </c>
+      <c r="T11" s="62" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="U11" s="63" t="n"/>
       <c r="V11" s="64" t="n"/>
       <c r="W11" s="62" t="inlineStr">
@@ -2840,29 +2908,77 @@
 Al fine di rendere non valido il token è necessario non valorizzare nel JWT il campo "purpose_of_use".</t>
         </is>
       </c>
-      <c r="F14" s="60" t="n"/>
-      <c r="G14" s="60" t="n"/>
-      <c r="H14" s="60" t="n"/>
-      <c r="I14" s="61" t="n"/>
+      <c r="F14" s="60" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="G14" s="60" t="inlineStr">
+        <is>
+          <t>2026-03-03 09:02:01</t>
+        </is>
+      </c>
+      <c r="H14" s="60" t="inlineStr">
+        <is>
+          <t>31b7c2d66522c545034d205231bd014a</t>
+        </is>
+      </c>
+      <c r="I14" s="61" t="inlineStr">
+        <is>
+          <t>UNKNOWN_WORKFLOW_ID</t>
+        </is>
+      </c>
       <c r="J14" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K14" s="62" t="inlineStr">
+        <is>
+          <t>Campo obbligatorio</t>
+        </is>
+      </c>
+      <c r="L14" s="62" t="n"/>
+      <c r="M14" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N14" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="O14" s="62" t="inlineStr">
+        <is>
+          <t>Il campo purpose_of_use non Ã¨ valorizzato</t>
+        </is>
+      </c>
+      <c r="P14" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q14" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R14" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="K14" s="62" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
-      <c r="L14" s="62" t="n"/>
-      <c r="M14" s="62" t="n"/>
-      <c r="N14" s="62" t="n"/>
-      <c r="O14" s="62" t="n"/>
-      <c r="P14" s="62" t="n"/>
-      <c r="Q14" s="62" t="n"/>
-      <c r="R14" s="62" t="n"/>
-      <c r="S14" s="62" t="n"/>
-      <c r="T14" s="62" t="n"/>
+      <c r="S14" s="62" t="inlineStr">
+        <is>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
+        </is>
+      </c>
+      <c r="T14" s="62" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="U14" s="63" t="n"/>
       <c r="V14" s="64" t="n"/>
       <c r="W14" s="62" t="inlineStr">
@@ -3135,29 +3251,77 @@
 Al fine di rendere non valido il token è necessario valorizzare il campo "action_id" con la stringa "TEST" (valore non ammesso).</t>
         </is>
       </c>
-      <c r="F19" s="60" t="n"/>
-      <c r="G19" s="60" t="n"/>
-      <c r="H19" s="60" t="n"/>
-      <c r="I19" s="61" t="n"/>
+      <c r="F19" s="60" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="G19" s="60" t="inlineStr">
+        <is>
+          <t>2026-03-03 09:02:00</t>
+        </is>
+      </c>
+      <c r="H19" s="60" t="inlineStr">
+        <is>
+          <t>97d09be041188fb796d6c547f0549b1f</t>
+        </is>
+      </c>
+      <c r="I19" s="61" t="inlineStr">
+        <is>
+          <t>UNKNOWN_WORKFLOW_ID</t>
+        </is>
+      </c>
       <c r="J19" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K19" s="62" t="inlineStr">
+        <is>
+          <t>Campo obbligatorio</t>
+        </is>
+      </c>
+      <c r="L19" s="62" t="n"/>
+      <c r="M19" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N19" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="O19" s="62" t="inlineStr">
+        <is>
+          <t>Il campo action_id non Ã¨ corretto</t>
+        </is>
+      </c>
+      <c r="P19" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q19" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R19" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="K19" s="62" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
-      <c r="L19" s="62" t="n"/>
-      <c r="M19" s="62" t="n"/>
-      <c r="N19" s="62" t="n"/>
-      <c r="O19" s="62" t="n"/>
-      <c r="P19" s="62" t="n"/>
-      <c r="Q19" s="62" t="n"/>
-      <c r="R19" s="62" t="n"/>
-      <c r="S19" s="62" t="n"/>
-      <c r="T19" s="62" t="n"/>
+      <c r="S19" s="62" t="inlineStr">
+        <is>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
+        </is>
+      </c>
+      <c r="T19" s="62" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="U19" s="63" t="n"/>
       <c r="V19" s="64" t="n"/>
       <c r="W19" s="62" t="inlineStr">
@@ -3312,29 +3476,77 @@
 Al fine di rendere non valido il token è necessario valorizzare il campo "action_id" con la stringa "TEST" (valore non ammesso).</t>
         </is>
       </c>
-      <c r="F22" s="60" t="n"/>
-      <c r="G22" s="60" t="n"/>
-      <c r="H22" s="60" t="n"/>
-      <c r="I22" s="61" t="n"/>
+      <c r="F22" s="60" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="G22" s="60" t="inlineStr">
+        <is>
+          <t>2026-03-03 09:02:03</t>
+        </is>
+      </c>
+      <c r="H22" s="60" t="inlineStr">
+        <is>
+          <t>c1c6ad99a691a319182336f8d8538a12</t>
+        </is>
+      </c>
+      <c r="I22" s="61" t="inlineStr">
+        <is>
+          <t>UNKNOWN_WORKFLOW_ID</t>
+        </is>
+      </c>
       <c r="J22" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K22" s="62" t="inlineStr">
+        <is>
+          <t>Campo obbligatorio</t>
+        </is>
+      </c>
+      <c r="L22" s="62" t="n"/>
+      <c r="M22" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N22" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="O22" s="62" t="inlineStr">
+        <is>
+          <t>Il campo action_id non Ã¨ corretto</t>
+        </is>
+      </c>
+      <c r="P22" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q22" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R22" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="K22" s="62" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
-      <c r="L22" s="62" t="n"/>
-      <c r="M22" s="62" t="n"/>
-      <c r="N22" s="62" t="n"/>
-      <c r="O22" s="62" t="n"/>
-      <c r="P22" s="62" t="n"/>
-      <c r="Q22" s="62" t="n"/>
-      <c r="R22" s="62" t="n"/>
-      <c r="S22" s="62" t="n"/>
-      <c r="T22" s="62" t="n"/>
+      <c r="S22" s="62" t="inlineStr">
+        <is>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
+        </is>
+      </c>
+      <c r="T22" s="62" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="U22" s="63" t="n"/>
       <c r="V22" s="64" t="n"/>
       <c r="W22" s="62" t="inlineStr">
@@ -3604,29 +3816,69 @@
 "ERRORE BLOCCANTE (SI/NO)", "ERRORE VISIBILE A UTENTE (SI/NO)", "MESSAGGIO DI ERRORE", "GESTITO IN BACKOFFICE (SI/NO)", " PRESENTE CODA DI RETRY AUTOMATICA PER L'INVIO DEL DOCUMENTO AL FSE SERVIZIO DI VALIDAZIONE DEL GATEWAY A SEGUITO DELLA RISOLUZIONE DELL'ERRORE (SI/NO)",  "INVIO MANUALE DEL DOCUMENTO AL FSE A SEGUITO DELLA RISOLUZIONE DELL'ERRORE (SI/NO)", "GESTIONE ERRORE".</t>
         </is>
       </c>
-      <c r="F27" s="60" t="n"/>
-      <c r="G27" s="60" t="n"/>
+      <c r="F27" s="60" t="inlineStr">
+        <is>
+          <t>26/02/2026</t>
+        </is>
+      </c>
+      <c r="G27" s="60" t="inlineStr">
+        <is>
+          <t>2026-02-26 18:38:30</t>
+        </is>
+      </c>
       <c r="H27" s="60" t="n"/>
       <c r="I27" s="61" t="n"/>
       <c r="J27" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K27" s="62" t="inlineStr">
+        <is>
+          <t>Campo obbligatorio</t>
+        </is>
+      </c>
+      <c r="L27" s="62" t="n"/>
+      <c r="M27" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N27" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="O27" s="62" t="inlineStr">
+        <is>
+          <t>HTTP/1.1 504 Gateway Timeout</t>
+        </is>
+      </c>
+      <c r="P27" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q27" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R27" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="K27" s="62" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
-      <c r="L27" s="62" t="n"/>
-      <c r="M27" s="62" t="n"/>
-      <c r="N27" s="62" t="n"/>
-      <c r="O27" s="62" t="n"/>
-      <c r="P27" s="62" t="n"/>
-      <c r="Q27" s="62" t="n"/>
-      <c r="R27" s="62" t="n"/>
-      <c r="S27" s="62" t="n"/>
-      <c r="T27" s="62" t="n"/>
+      <c r="S27" s="62" t="inlineStr">
+        <is>
+          <t>In caso di timeout viene notificato all'utente e il documento viene gestito tramite coda di retry fino al ripristino del servizio.</t>
+        </is>
+      </c>
+      <c r="T27" s="62" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="U27" s="63" t="inlineStr">
         <is>
           <t>SI</t>
@@ -3784,29 +4036,69 @@
 "ERRORE BLOCCANTE (SI/NO)", "ERRORE VISIBILE A UTENTE (SI/NO)", "MESSAGGIO DI ERRORE", "GESTITO IN BACKOFFICE (SI/NO)", " PRESENTE CODA DI RETRY AUTOMATICA PER L'INVIO DEL DOCUMENTO AL FSE SERVIZIO DI VALIDAZIONE DEL GATEWAY A SEGUITO DELLA RISOLUZIONE DELL'ERRORE (SI/NO)",  "INVIO MANUALE DEL DOCUMENTO AL FSE A SEGUITO DELLA RISOLUZIONE DELL'ERRORE (SI/NO)", "GESTIONE ERRORE".</t>
         </is>
       </c>
-      <c r="F30" s="60" t="n"/>
-      <c r="G30" s="60" t="n"/>
+      <c r="F30" s="60" t="inlineStr">
+        <is>
+          <t>26/02/2026</t>
+        </is>
+      </c>
+      <c r="G30" s="60" t="inlineStr">
+        <is>
+          <t>2026-02-26 18:38:30</t>
+        </is>
+      </c>
       <c r="H30" s="60" t="n"/>
       <c r="I30" s="61" t="n"/>
       <c r="J30" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="K30" s="62" t="inlineStr">
+        <is>
+          <t>Campo obbligatorio</t>
+        </is>
+      </c>
+      <c r="L30" s="62" t="n"/>
+      <c r="M30" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N30" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="O30" s="62" t="inlineStr">
+        <is>
+          <t>HTTP/1.1 504 Gateway Timeout</t>
+        </is>
+      </c>
+      <c r="P30" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q30" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R30" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="K30" s="62" t="inlineStr">
-        <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
-      <c r="L30" s="62" t="n"/>
-      <c r="M30" s="62" t="n"/>
-      <c r="N30" s="62" t="n"/>
-      <c r="O30" s="62" t="n"/>
-      <c r="P30" s="62" t="n"/>
-      <c r="Q30" s="62" t="n"/>
-      <c r="R30" s="62" t="n"/>
-      <c r="S30" s="62" t="n"/>
-      <c r="T30" s="62" t="n"/>
+      <c r="S30" s="62" t="inlineStr">
+        <is>
+          <t>In caso di timeout viene notificato all'utente e il documento viene gestito tramite coda di retry fino al ripristino del servizio.</t>
+        </is>
+      </c>
+      <c r="T30" s="62" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="U30" s="63" t="inlineStr">
         <is>
           <t>SI</t>
@@ -4094,8 +4386,16 @@
           <t>2026-02-26 18:37:51</t>
         </is>
       </c>
-      <c r="H35" s="60" t="inlineStr"/>
-      <c r="I35" s="61" t="inlineStr"/>
+      <c r="H35" s="60" t="inlineStr">
+        <is>
+          <t>738ab0b919983bfa9f21f0ada3a0a084</t>
+        </is>
+      </c>
+      <c r="I35" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.bca91958642e9381485555f996bfa4d7a88762d1e9f3ebfe6ec9783e1415303d.33ed0fd4f8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J35" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -4115,27 +4415,27 @@
       </c>
       <c r="O35" s="62" t="inlineStr">
         <is>
-          <t>HTTP 403 - Errore validazione CDA2</t>
+          <t>JWT payload: Person id presente nel JWT differente dal codice fiscale del paziente previsto sul CDA</t>
         </is>
       </c>
       <c r="P35" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q35" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R35" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q35" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R35" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S35" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T35" s="62" t="inlineStr">
@@ -4186,8 +4486,16 @@
           <t>2026-02-26 18:37:53</t>
         </is>
       </c>
-      <c r="H36" s="60" t="inlineStr"/>
-      <c r="I36" s="61" t="inlineStr"/>
+      <c r="H36" s="60" t="inlineStr">
+        <is>
+          <t>96a34b52ad35b1f2e17548d4846fe01f</t>
+        </is>
+      </c>
+      <c r="I36" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.bca91958642e9381485555f996bfa4d7a88762d1e9f3ebfe6ec9783e1415303d.f6cb0aa608^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J36" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -4207,27 +4515,27 @@
       </c>
       <c r="O36" s="62" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>ERROR: -1,-1 cvc-complex-type.2.4.a: Invalid content was found starting with element '{"urn:hl7-org:v3":addr}'. One of '{"urn:hl7-org:v3":providerOrganization}' is expected.</t>
         </is>
       </c>
       <c r="P36" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q36" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R36" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q36" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R36" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S36" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T36" s="62" t="inlineStr">
@@ -4278,8 +4586,16 @@
           <t>2026-02-26 18:37:54</t>
         </is>
       </c>
-      <c r="H37" s="60" t="inlineStr"/>
-      <c r="I37" s="61" t="inlineStr"/>
+      <c r="H37" s="60" t="inlineStr">
+        <is>
+          <t>901839e410e3bfc9245d2874b1fae7f9</t>
+        </is>
+      </c>
+      <c r="I37" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.bca91958642e9381485555f996bfa4d7a88762d1e9f3ebfe6ec9783e1415303d.d92a0acdc4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J37" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -4299,27 +4615,27 @@
       </c>
       <c r="O37" s="62" t="inlineStr">
         <is>
-          <t>HTTP 422 - Errore validazione CDA2</t>
+          <t>[ERRORE-15| L'elemento ClinicalDocument/recordTaget/patientRole/patient/name DEVE riportare gli elementi 'given' e 'family']</t>
         </is>
       </c>
       <c r="P37" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q37" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R37" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q37" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R37" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S37" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T37" s="62" t="inlineStr">
@@ -4370,8 +4686,16 @@
           <t>2026-02-26 18:37:55</t>
         </is>
       </c>
-      <c r="H38" s="60" t="inlineStr"/>
-      <c r="I38" s="61" t="inlineStr"/>
+      <c r="H38" s="60" t="inlineStr">
+        <is>
+          <t>bf51d6d63997e68a2d808e13c7053939</t>
+        </is>
+      </c>
+      <c r="I38" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.bca91958642e9381485555f996bfa4d7a88762d1e9f3ebfe6ec9783e1415303d.85de4c3378^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J38" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -4391,27 +4715,27 @@
       </c>
       <c r="O38" s="62" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>Almeno uno dei seguenti vocaboli non Ã¨ censito: [CodeSystem: 2.16.840.1.113883.5.1 v2.1.0, Codes: X]</t>
         </is>
       </c>
       <c r="P38" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q38" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R38" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q38" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R38" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S38" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T38" s="62" t="inlineStr">
@@ -4462,8 +4786,16 @@
           <t>2026-02-26 18:37:57</t>
         </is>
       </c>
-      <c r="H39" s="60" t="inlineStr"/>
-      <c r="I39" s="61" t="inlineStr"/>
+      <c r="H39" s="60" t="inlineStr">
+        <is>
+          <t>b54323677e22b4c3ce5029c770a13b8a</t>
+        </is>
+      </c>
+      <c r="I39" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.bca91958642e9381485555f996bfa4d7a88762d1e9f3ebfe6ec9783e1415303d.a03482323c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J39" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -4483,27 +4815,27 @@
       </c>
       <c r="O39" s="62" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>ERROR: -1,-1 cvc-complex-type.2.4.b: The content of element 'order' is not complete. One of '{"urn:hl7-org:v3":realmCode, "urn:hl7-org:v3":typeId, "urn:hl7-org:v3":templateId, "urn:hl7-org:v3":id}' is expected.</t>
         </is>
       </c>
       <c r="P39" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q39" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R39" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q39" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R39" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S39" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T39" s="62" t="inlineStr">
@@ -4554,8 +4886,16 @@
           <t>2026-02-26 18:37:58</t>
         </is>
       </c>
-      <c r="H40" s="60" t="inlineStr"/>
-      <c r="I40" s="61" t="inlineStr"/>
+      <c r="H40" s="60" t="inlineStr">
+        <is>
+          <t>99d7286aaf4b2ecfb7142b9efb79aa32</t>
+        </is>
+      </c>
+      <c r="I40" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.bca91958642e9381485555f996bfa4d7a88762d1e9f3ebfe6ec9783e1415303d.27bdaa4598^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J40" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -4575,27 +4915,48 @@
       </c>
       <c r="O40" s="62" t="inlineStr">
         <is>
-          <t>HTTP 422 - Errore validazione CDA2</t>
+          <t>[ERRORE-b1| L'elemento code della section DEVE essere valorizzato con uno dei seguenti codici LOINC individuati:
+						18717-9 BANCA DEL SANGUE
+						18718-7 MARCATORI CELLULARI 
+						18719-5 CHIMICA
+						18720-3	COAGULAZIONE
+						18721-1 MONITORAGGIO TERAPEUTICO DEI FARMACI
+						18722-9 FERTILITÃ€
+						18723-7 EMATOLOGIA
+						18724-5 HLA
+						18725-2 MICROBIOLOGIA
+						18727-8 SEROLOGIA
+						18728-6 TOSSICOLOGIA
+						18729-4 ESAMI DELLE URINE
+						18767-4 EMOGASANALISI
+						18768-2 CONTE CELLULARE+DIFFERENZIALE
+						18769-0 SUSCETTIBILITÃ€ ANTIMICROBICA
+						26435-8 PATOLOGIA MOLECOLARE
+						26436-6 ESAMI DI LABORATORIO
+						26437-4 TEST DI SENSIBILITÃ€ A SOSTANZE CHIMICHE
+						26438-2 CITOLOGIA
+						18716-1 ALLERGOLOGIA
+						26439-0 PATOLOGIA CHIRURGICA]</t>
         </is>
       </c>
       <c r="P40" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q40" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R40" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q40" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R40" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S40" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T40" s="62" t="inlineStr">
@@ -4646,8 +5007,16 @@
           <t>2026-02-26 18:37:59</t>
         </is>
       </c>
-      <c r="H41" s="60" t="inlineStr"/>
-      <c r="I41" s="61" t="inlineStr"/>
+      <c r="H41" s="60" t="inlineStr">
+        <is>
+          <t>4419fa599121b2d45e44c9add6cad697</t>
+        </is>
+      </c>
+      <c r="I41" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.bca91958642e9381485555f996bfa4d7a88762d1e9f3ebfe6ec9783e1415303d.4c93ea7dfe^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J41" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -4667,27 +5036,27 @@
       </c>
       <c r="O41" s="62" t="inlineStr">
         <is>
-          <t>HTTP 422 - Errore validazione CDA2</t>
+          <t>[ERRORE-b11| L'elemento specimen/specimenRole/specimenPlayingEntity deve contenere l'elemento 'code'],[ERRORE-b11| L'elemento specimen/specimenRole/specimenPlayingEntity deve contenere l'elemento 'code']</t>
         </is>
       </c>
       <c r="P41" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q41" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R41" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q41" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R41" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S41" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T41" s="62" t="inlineStr">
@@ -4738,8 +5107,16 @@
           <t>2026-02-26 18:38:01</t>
         </is>
       </c>
-      <c r="H42" s="60" t="inlineStr"/>
-      <c r="I42" s="61" t="inlineStr"/>
+      <c r="H42" s="60" t="inlineStr">
+        <is>
+          <t>877eac0cb0c42310ffee480dd6a30ced</t>
+        </is>
+      </c>
+      <c r="I42" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.bca91958642e9381485555f996bfa4d7a88762d1e9f3ebfe6ec9783e1415303d.869a8829cd^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J42" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -4759,27 +5136,28 @@
       </c>
       <c r="O42" s="62" t="inlineStr">
         <is>
-          <t>HTTP 422 - Errore validazione CDA2</t>
+          <t>[ERRORE-b19| LÂ’elemento organizer di tipo 'BATTERY' (@classCode='BATTERY') DEVE contenere lÂ’elemento organizer/code.
+			]</t>
         </is>
       </c>
       <c r="P42" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q42" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R42" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q42" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R42" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S42" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T42" s="62" t="inlineStr">
@@ -5390,8 +5768,16 @@
           <t>2026-02-26 18:38:08</t>
         </is>
       </c>
-      <c r="H53" s="60" t="inlineStr"/>
-      <c r="I53" s="61" t="inlineStr"/>
+      <c r="H53" s="60" t="inlineStr">
+        <is>
+          <t>3e819a83016dd3b6019276ee2888d792</t>
+        </is>
+      </c>
+      <c r="I53" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.ea14ba098e0194e3e55227022cb22641378e7754eb8c2dd76a91d41f7fea3b9e.e1a6c0a41b^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J53" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -5411,27 +5797,27 @@
       </c>
       <c r="O53" s="62" t="inlineStr">
         <is>
-          <t>HTTP 403 - Errore validazione CDA2</t>
+          <t>JWT payload: Person id presente nel JWT differente dal codice fiscale del paziente previsto sul CDA</t>
         </is>
       </c>
       <c r="P53" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q53" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R53" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q53" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R53" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S53" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T53" s="62" t="inlineStr">
@@ -5482,8 +5868,16 @@
           <t>2026-02-26 18:38:10</t>
         </is>
       </c>
-      <c r="H54" s="60" t="inlineStr"/>
-      <c r="I54" s="61" t="inlineStr"/>
+      <c r="H54" s="60" t="inlineStr">
+        <is>
+          <t>3e1ae653642bb33859e873994211cdd1</t>
+        </is>
+      </c>
+      <c r="I54" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.76388e42d50d2e40a09aa205b48d619f7e3042d1a68a3753f0f6eac8da7ee467.e52edf9ed4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J54" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -5503,27 +5897,27 @@
       </c>
       <c r="O54" s="62" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>ERROR: -1,-1 cvc-complex-type.2.4.a: Invalid content was found starting with element '{"urn:hl7-org:v3":addr}'. One of '{"urn:hl7-org:v3":providerOrganization}' is expected.</t>
         </is>
       </c>
       <c r="P54" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q54" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R54" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q54" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R54" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S54" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T54" s="62" t="inlineStr">
@@ -5574,8 +5968,16 @@
           <t>2026-02-26 18:38:11</t>
         </is>
       </c>
-      <c r="H55" s="60" t="inlineStr"/>
-      <c r="I55" s="61" t="inlineStr"/>
+      <c r="H55" s="60" t="inlineStr">
+        <is>
+          <t>710becbd19657c9c1c587fa146e84f9c</t>
+        </is>
+      </c>
+      <c r="I55" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.e3569ff22cf79a9150d70d439204a1ad50f2b01338697a3ad06dfe9bdc52843a.702c41c177^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J55" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -5595,27 +5997,27 @@
       </c>
       <c r="O55" s="62" t="inlineStr">
         <is>
-          <t>HTTP 422 - Errore validazione CDA2</t>
+          <t>[ERRORE-14| L'elemento ClinicalDocument/recordTaget/patientRole/patient/name DEVE riportare gli elementi 'given' e 'family']</t>
         </is>
       </c>
       <c r="P55" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q55" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R55" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q55" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R55" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S55" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T55" s="62" t="inlineStr">
@@ -5666,8 +6068,16 @@
           <t>2026-02-26 18:38:13</t>
         </is>
       </c>
-      <c r="H56" s="60" t="inlineStr"/>
-      <c r="I56" s="61" t="inlineStr"/>
+      <c r="H56" s="60" t="inlineStr">
+        <is>
+          <t>9a268af24127d69c3646bf5c869f70db</t>
+        </is>
+      </c>
+      <c r="I56" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.7c28886e9d7374a4caa00733f99a385665138c427282adc8cfc011c5be745b0c.31fa7af2cf^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J56" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -5687,27 +6097,27 @@
       </c>
       <c r="O56" s="62" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>Almeno uno dei seguenti vocaboli non Ã¨ censito: [CodeSystem: 2.16.840.1.113883.5.1 v2.1.0, Codes: NB]</t>
         </is>
       </c>
       <c r="P56" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q56" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R56" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q56" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R56" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S56" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T56" s="62" t="inlineStr">
@@ -5758,8 +6168,16 @@
           <t>2026-02-26 18:38:14</t>
         </is>
       </c>
-      <c r="H57" s="60" t="inlineStr"/>
-      <c r="I57" s="61" t="inlineStr"/>
+      <c r="H57" s="60" t="inlineStr">
+        <is>
+          <t>d80029c381c12df8ee428ab194f642f5</t>
+        </is>
+      </c>
+      <c r="I57" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.7df6ebadd13a618ec3279ff29f38a5620c2b007e05f30bbf9f3886f499a970a1.75c6303042^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J57" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -5779,27 +6197,27 @@
       </c>
       <c r="O57" s="62" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>ERROR: -1,-1 cvc-complex-type.2.4.d: Invalid content was found starting with element 'participant'. No child element is expected at this point.</t>
         </is>
       </c>
       <c r="P57" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q57" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R57" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q57" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R57" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S57" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T57" s="62" t="inlineStr">
@@ -5850,8 +6268,16 @@
           <t>2026-02-26 18:38:15</t>
         </is>
       </c>
-      <c r="H58" s="60" t="inlineStr"/>
-      <c r="I58" s="61" t="inlineStr"/>
+      <c r="H58" s="60" t="inlineStr">
+        <is>
+          <t>ce65d5fb00c941b816de74377a9455e4</t>
+        </is>
+      </c>
+      <c r="I58" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.8243d8f6719687e5ab7a4aea230bae977419f6d1e0c28717305abba98abaf3ce.e092523357^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J58" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -5871,27 +6297,27 @@
       </c>
       <c r="O58" s="62" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>ERROR: -1,-1 cvc-complex-type.2.4.b: The content of element 'order' is not complete. One of '{"urn:hl7-org:v3":realmCode, "urn:hl7-org:v3":typeId, "urn:hl7-org:v3":templateId, "urn:hl7-org:v3":id}' is expected.</t>
         </is>
       </c>
       <c r="P58" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q58" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R58" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q58" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R58" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S58" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T58" s="62" t="inlineStr">
@@ -5942,8 +6368,16 @@
           <t>2026-02-26 18:38:16</t>
         </is>
       </c>
-      <c r="H59" s="60" t="inlineStr"/>
-      <c r="I59" s="61" t="inlineStr"/>
+      <c r="H59" s="60" t="inlineStr">
+        <is>
+          <t>f411a5d509797f0b9ade956cf446a96c</t>
+        </is>
+      </c>
+      <c r="I59" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.6e6bc3733dcdf10c57c1d4adf2d330aff551564f93fb78a376bf8962e4955541.ab138581cf^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J59" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -5963,27 +6397,27 @@
       </c>
       <c r="O59" s="62" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>ERROR: -1,-1 cvc-complex-type.2.4.a: Invalid content was found starting with element '{"urn:hl7-org:v3":statusCode}'. One of '{"urn:hl7-org:v3":realmCode, "urn:hl7-org:v3":typeId, "urn:hl7-org:v3":templateId, "urn:hl7-org:v3":id, "urn:hl7-org:v3":code}' is expected.</t>
         </is>
       </c>
       <c r="P59" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q59" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R59" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q59" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R59" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S59" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T59" s="62" t="inlineStr">
@@ -6034,8 +6468,16 @@
           <t>2026-02-26 18:38:18</t>
         </is>
       </c>
-      <c r="H60" s="60" t="inlineStr"/>
-      <c r="I60" s="61" t="inlineStr"/>
+      <c r="H60" s="60" t="inlineStr">
+        <is>
+          <t>f1c187758d00a35240cd82e55a989158</t>
+        </is>
+      </c>
+      <c r="I60" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.ba95e5c839949970731d9d7fc25d372f6dcd9892ea08396c851538e935610020.754b9b3ecc^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J60" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -6055,27 +6497,27 @@
       </c>
       <c r="O60" s="62" t="inlineStr">
         <is>
-          <t>HTTP 422 - Errore validazione CDA2</t>
+          <t>[ERRORE-b4| Sezione Referto: DEVE essere presente la sezione "Referto".],[ERRORE-b5| Sezione Referto: La sezione deve contenere l'elemento 'text'.]</t>
         </is>
       </c>
       <c r="P60" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q60" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R60" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q60" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R60" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S60" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T60" s="62" t="inlineStr">
@@ -6126,8 +6568,16 @@
           <t>2026-02-26 18:38:19</t>
         </is>
       </c>
-      <c r="H61" s="60" t="inlineStr"/>
-      <c r="I61" s="61" t="inlineStr"/>
+      <c r="H61" s="60" t="inlineStr">
+        <is>
+          <t>b4915a86dc2b9a8abd90b0de2382329b</t>
+        </is>
+      </c>
+      <c r="I61" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.1582e4d3da50d728b3745e95c5541e4646560e2a77d56af4521691016e3b5707.bbbd91f062^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J61" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -6147,27 +6597,27 @@
       </c>
       <c r="O61" s="62" t="inlineStr">
         <is>
-          <t>HTTP 422 - Errore validazione CDA2</t>
+          <t>[ERRORE-b13| Sezione Precedenti Esami Eseguiti: La section deve contenere l'elemento 'text'.]</t>
         </is>
       </c>
       <c r="P61" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q61" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R61" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q61" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R61" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S61" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T61" s="62" t="inlineStr">
@@ -6218,8 +6668,16 @@
           <t>2026-02-26 18:38:20</t>
         </is>
       </c>
-      <c r="H62" s="60" t="inlineStr"/>
-      <c r="I62" s="61" t="inlineStr"/>
+      <c r="H62" s="60" t="inlineStr">
+        <is>
+          <t>7e7434bfc75aa6bcb4914f5020eae1e2</t>
+        </is>
+      </c>
+      <c r="I62" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.74a1f8f05dbdcf11890edee3f4c20fbdfe335132a30c756bcbd9df89146fb22b.5016666c34^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J62" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -6239,27 +6697,27 @@
       </c>
       <c r="O62" s="62" t="inlineStr">
         <is>
-          <t>HTTP 422 - Errore validazione CDA2</t>
+          <t>[ERRORE-b7| Sezione Dicom Object Catalog: La sezione deve avere l'elemento 'entry' di tipo 'act'.]</t>
         </is>
       </c>
       <c r="P62" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q62" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R62" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q62" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R62" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S62" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T62" s="62" t="inlineStr">
@@ -6310,8 +6768,16 @@
           <t>2026-02-26 18:38:22</t>
         </is>
       </c>
-      <c r="H63" s="60" t="inlineStr"/>
-      <c r="I63" s="61" t="inlineStr"/>
+      <c r="H63" s="60" t="inlineStr">
+        <is>
+          <t>cf96b342b299a9a127cc23bff88bcf60</t>
+        </is>
+      </c>
+      <c r="I63" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.d7d5b9a29951eb390440b77925eb9bfc992df0115808f61461d7b780e15ee562.2ede670ade^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J63" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -6331,27 +6797,27 @@
       </c>
       <c r="O63" s="62" t="inlineStr">
         <is>
-          <t>HTTP 422 - Errore validazione CDA2</t>
+          <t>[ERRORE-b22| Sezione Storia Clinica: L'elemento entry/observation/effectiveTime deve essere presente e deve avere l'elemento 'low' valorizzato.]</t>
         </is>
       </c>
       <c r="P63" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q63" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R63" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q63" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R63" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S63" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T63" s="62" t="inlineStr">
@@ -6402,8 +6868,16 @@
           <t>2026-02-26 18:38:23</t>
         </is>
       </c>
-      <c r="H64" s="60" t="inlineStr"/>
-      <c r="I64" s="61" t="inlineStr"/>
+      <c r="H64" s="60" t="inlineStr">
+        <is>
+          <t>24c3a497afc58996a1d2446191622c41</t>
+        </is>
+      </c>
+      <c r="I64" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.99492cfff4da413aad813dd7283842da2d68b187541fd27ff1295b59c012c854.cd86476daa^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J64" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -6423,27 +6897,27 @@
       </c>
       <c r="O64" s="62" t="inlineStr">
         <is>
-          <t>HTTP 422 - Errore validazione CDA2</t>
+          <t>[ERRORE-b26| Sezione Storia Clinica: La entry/organizer deve avere un elemento subject/relatedSubject il quale deve contenere l'elemento 'code'. ]</t>
         </is>
       </c>
       <c r="P64" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q64" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R64" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q64" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R64" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S64" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T64" s="62" t="inlineStr">
@@ -6494,8 +6968,16 @@
           <t>2026-02-26 18:38:24</t>
         </is>
       </c>
-      <c r="H65" s="60" t="inlineStr"/>
-      <c r="I65" s="61" t="inlineStr"/>
+      <c r="H65" s="60" t="inlineStr">
+        <is>
+          <t>0af677b5cd3551ab7f3b88c4d07da1f4</t>
+        </is>
+      </c>
+      <c r="I65" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.58f5a1311a3a464d152b8d42c234bb3731e355def108e854ecd17f613f88a4ff.d4cab979a7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J65" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -6515,27 +6997,27 @@
       </c>
       <c r="O65" s="62" t="inlineStr">
         <is>
-          <t>HTTP 422 - Errore validazione CDA2</t>
+          <t>[ERRORE-b53| Sotto sezione Allergie: I'elemento entry/act/entryRelationship/observation/effectiveTime deve avere valorizzato l'elemento 'low'.]</t>
         </is>
       </c>
       <c r="P65" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q65" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R65" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q65" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R65" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S65" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T65" s="62" t="inlineStr">
@@ -6586,8 +7068,16 @@
           <t>2026-02-26 18:38:25</t>
         </is>
       </c>
-      <c r="H66" s="60" t="inlineStr"/>
-      <c r="I66" s="61" t="inlineStr"/>
+      <c r="H66" s="60" t="inlineStr">
+        <is>
+          <t>e1acb2af31574870ea988fbc650c047b</t>
+        </is>
+      </c>
+      <c r="I66" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.b274fc9da5cffae1695615d3175e0ae368154bc151c93b518e64701960e6af48.21e443ee67^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J66" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -6607,27 +7097,27 @@
       </c>
       <c r="O66" s="62" t="inlineStr">
         <is>
-          <t>HTTP 422 - Errore validazione CDA2</t>
+          <t>[ERRORE-b57| Sotto sezione Allergie: L'elemento entryRelationship/observation (Descrizione Agente) deve avere almeno un elemento 'participant' che dettaglia l'agente scatenante.]</t>
         </is>
       </c>
       <c r="P66" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q66" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R66" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q66" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R66" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S66" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T66" s="62" t="inlineStr">
@@ -6678,8 +7168,16 @@
           <t>2026-02-26 18:38:27</t>
         </is>
       </c>
-      <c r="H67" s="60" t="inlineStr"/>
-      <c r="I67" s="61" t="inlineStr"/>
+      <c r="H67" s="60" t="inlineStr">
+        <is>
+          <t>bf286f0592f4583c89e1d0b109abe861</t>
+        </is>
+      </c>
+      <c r="I67" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.5d698c31f4d534430106b31236ffcb93711e1ae5acb6e7f189623a01ac0abf65.2946d1a08d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J67" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -6699,27 +7197,27 @@
       </c>
       <c r="O67" s="62" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>Almeno uno dei seguenti vocaboli non Ã¨ censito: [CodeSystem: 2.16.840.1.113883.6.103, Codes: CODICE_ERRATO_999]</t>
         </is>
       </c>
       <c r="P67" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q67" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R67" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q67" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R67" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S67" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T67" s="62" t="inlineStr">
@@ -6770,8 +7268,16 @@
           <t>2026-02-26 18:38:28</t>
         </is>
       </c>
-      <c r="H68" s="60" t="inlineStr"/>
-      <c r="I68" s="61" t="inlineStr"/>
+      <c r="H68" s="60" t="inlineStr">
+        <is>
+          <t>a29494d512e6ebbbd4f1940871b5c4c2</t>
+        </is>
+      </c>
+      <c r="I68" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.9a03a97ac833ddb83eca6797ce8021ae4e2781cd601607af73a33c216cfa31a2.f1e98b149d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J68" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -6791,27 +7297,27 @@
       </c>
       <c r="O68" s="62" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>ERROR: -1,-1 cvc-complex-type.2.4.d: Invalid content was found starting with element 'documentationOf'. No child element is expected at this point.</t>
         </is>
       </c>
       <c r="P68" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q68" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R68" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q68" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R68" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S68" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T68" s="62" t="inlineStr">
@@ -11176,10 +11682,14 @@
       </c>
       <c r="K146" s="62" t="inlineStr">
         <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
-      <c r="L146" s="62" t="n"/>
+          <t>Altro (specificare)</t>
+        </is>
+      </c>
+      <c r="L146" s="62" t="inlineStr">
+        <is>
+          <t>Non gestiamo le trasfusioni</t>
+        </is>
+      </c>
       <c r="M146" s="62" t="n"/>
       <c r="N146" s="62" t="n"/>
       <c r="O146" s="62" t="n"/>
@@ -11187,7 +11697,11 @@
       <c r="Q146" s="62" t="n"/>
       <c r="R146" s="62" t="n"/>
       <c r="S146" s="62" t="n"/>
-      <c r="T146" s="62" t="n"/>
+      <c r="T146" s="62" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="U146" s="63" t="n"/>
       <c r="V146" s="64" t="n"/>
       <c r="W146" s="62" t="inlineStr">
@@ -11233,10 +11747,14 @@
       </c>
       <c r="K147" s="62" t="inlineStr">
         <is>
-          <t>Campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
-        </is>
-      </c>
-      <c r="L147" s="62" t="n"/>
+          <t>Altro (specificare)</t>
+        </is>
+      </c>
+      <c r="L147" s="62" t="inlineStr">
+        <is>
+          <t>Non gestiamo le trasfusioni</t>
+        </is>
+      </c>
       <c r="M147" s="62" t="n"/>
       <c r="N147" s="62" t="n"/>
       <c r="O147" s="62" t="n"/>
@@ -11244,7 +11762,11 @@
       <c r="Q147" s="62" t="n"/>
       <c r="R147" s="62" t="n"/>
       <c r="S147" s="62" t="n"/>
-      <c r="T147" s="62" t="n"/>
+      <c r="T147" s="62" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="U147" s="63" t="n"/>
       <c r="V147" s="64" t="n"/>
       <c r="W147" s="62" t="inlineStr">
@@ -12419,7 +12941,7 @@
       </c>
       <c r="H168" s="60" t="inlineStr">
         <is>
-          <t>74a1f8f05dbdcf11890edee3f4c20fbdfe335132a30c756bcbd9df89146fb22b</t>
+          <t>87b13c8ca60a19a4f2d511e6dfb9de24</t>
         </is>
       </c>
       <c r="I168" s="61" t="inlineStr">
@@ -12434,12 +12956,32 @@
       </c>
       <c r="K168" s="62" t="n"/>
       <c r="L168" s="62" t="n"/>
-      <c r="M168" s="62" t="n"/>
-      <c r="N168" s="62" t="n"/>
+      <c r="M168" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="N168" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="O168" s="62" t="n"/>
-      <c r="P168" s="62" t="n"/>
-      <c r="Q168" s="62" t="n"/>
-      <c r="R168" s="62" t="n"/>
+      <c r="P168" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q168" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R168" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="S168" s="62" t="n"/>
       <c r="T168" s="62" t="inlineStr">
         <is>
@@ -12937,8 +13479,16 @@
           <t>2026-02-26 18:38:29</t>
         </is>
       </c>
-      <c r="H177" s="57" t="inlineStr"/>
-      <c r="I177" s="57" t="inlineStr"/>
+      <c r="H177" s="57" t="inlineStr">
+        <is>
+          <t>89608007be46962e7dee4476021019ac</t>
+        </is>
+      </c>
+      <c r="I177" s="57" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.71584c703de07f3b50d646b1ae7caf4e359eb549336dead486459ac15456c4fe.319ec7eec0^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J177" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -12958,27 +13508,27 @@
       </c>
       <c r="O177" s="57" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>ERROR: -1,-1 cvc-complex-type.2.4.a: Invalid content was found starting with element '{"urn:hl7-org:v3":languageCode}'. One of '{"urn:hl7-org:v3":confidentialityCode}' is expected.</t>
         </is>
       </c>
       <c r="P177" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q177" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R177" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q177" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R177" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S177" s="57" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T177" s="62" t="inlineStr">
@@ -13197,8 +13747,16 @@
           <t>2026-02-26 18:38:02</t>
         </is>
       </c>
-      <c r="H181" s="57" t="inlineStr"/>
-      <c r="I181" s="57" t="inlineStr"/>
+      <c r="H181" s="57" t="inlineStr">
+        <is>
+          <t>c47bc007f1022aa5e609ddae19f9a169</t>
+        </is>
+      </c>
+      <c r="I181" s="57" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.bca91958642e9381485555f996bfa4d7a88762d1e9f3ebfe6ec9783e1415303d.90d54c3c22^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J181" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -13218,27 +13776,27 @@
       </c>
       <c r="O181" s="57" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>ERROR: -1,-1 cvc-complex-type.2.4.a: Invalid content was found starting with element '{"urn:hl7-org:v3":languageCode}'. One of '{"urn:hl7-org:v3":confidentialityCode}' is expected.</t>
         </is>
       </c>
       <c r="P181" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q181" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R181" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q181" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R181" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S181" s="57" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T181" s="62" t="inlineStr">
@@ -13515,7 +14073,7 @@
       </c>
       <c r="H186" s="60" t="inlineStr">
         <is>
-          <t>230ffe4d6cdd2160bb19c431b3a4593a3ffd683f64b7405d3e4d4e5f82ec0234</t>
+          <t>460ff6c1888c20b10bba793b9398a617</t>
         </is>
       </c>
       <c r="I186" s="61" t="inlineStr">
@@ -13530,12 +14088,32 @@
       </c>
       <c r="K186" s="62" t="n"/>
       <c r="L186" s="62" t="n"/>
-      <c r="M186" s="62" t="n"/>
-      <c r="N186" s="62" t="n"/>
+      <c r="M186" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="N186" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="O186" s="62" t="n"/>
-      <c r="P186" s="62" t="n"/>
-      <c r="Q186" s="62" t="n"/>
-      <c r="R186" s="62" t="n"/>
+      <c r="P186" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q186" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R186" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="S186" s="62" t="n"/>
       <c r="T186" s="62" t="inlineStr">
         <is>
@@ -13587,7 +14165,7 @@
       </c>
       <c r="H187" s="60" t="inlineStr">
         <is>
-          <t>2346f2c34297d8cdab56fd4b47e8a90f1948d30be64d8293e67dabd0a737b9e6</t>
+          <t>3a5d92f200e2ae1bfb0e2f4e8f4593f9</t>
         </is>
       </c>
       <c r="I187" s="61" t="inlineStr">
@@ -13602,12 +14180,32 @@
       </c>
       <c r="K187" s="62" t="n"/>
       <c r="L187" s="62" t="n"/>
-      <c r="M187" s="62" t="n"/>
-      <c r="N187" s="62" t="n"/>
+      <c r="M187" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="N187" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="O187" s="62" t="n"/>
-      <c r="P187" s="62" t="n"/>
-      <c r="Q187" s="62" t="n"/>
-      <c r="R187" s="62" t="n"/>
+      <c r="P187" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q187" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R187" s="62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="S187" s="62" t="n"/>
       <c r="T187" s="62" t="inlineStr">
         <is>
@@ -13657,8 +14255,16 @@
           <t>2026-02-26 18:38:03</t>
         </is>
       </c>
-      <c r="H188" s="60" t="inlineStr"/>
-      <c r="I188" s="61" t="inlineStr"/>
+      <c r="H188" s="60" t="inlineStr">
+        <is>
+          <t>ebc0371cbb48686d971c7e10fb2abae5</t>
+        </is>
+      </c>
+      <c r="I188" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.bca91958642e9381485555f996bfa4d7a88762d1e9f3ebfe6ec9783e1415303d.69ab10264d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J188" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -13678,27 +14284,27 @@
       </c>
       <c r="O188" s="62" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>Almeno uno dei seguenti vocaboli non Ã¨ censito: [CodeSystem: 2.16.840.1.113883.5.7 v2.1.0, Codes: INVALID_PRIORITY]</t>
         </is>
       </c>
       <c r="P188" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q188" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R188" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q188" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R188" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S188" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T188" s="62" t="inlineStr">
@@ -13749,8 +14355,16 @@
           <t>2026-02-26 18:38:30</t>
         </is>
       </c>
-      <c r="H189" s="60" t="inlineStr"/>
-      <c r="I189" s="61" t="inlineStr"/>
+      <c r="H189" s="60" t="inlineStr">
+        <is>
+          <t>6c81b91fd426d78ce5fb8229de210b04</t>
+        </is>
+      </c>
+      <c r="I189" s="61" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.6ebfdb900a10479d3bbf514e2562c0430c0eb7602656c5ec1dabbcfc08b820a5.0457f4ca1b^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J189" s="62" t="inlineStr">
         <is>
           <t>SI</t>
@@ -13770,27 +14384,27 @@
       </c>
       <c r="O189" s="62" t="inlineStr">
         <is>
-          <t>HTTP 400 - Errore validazione CDA2</t>
+          <t>Almeno uno dei seguenti vocaboli non Ã¨ censito: [CodeSystem: 2.16.840.1.113883.5.7 v2.1.0, Codes: INVALID_PRIORITY]</t>
         </is>
       </c>
       <c r="P189" s="62" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q189" s="62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R189" s="62" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q189" s="62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R189" s="62" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S189" s="62" t="inlineStr">
         <is>
-          <t>Il sistema blocca la pubblicazione e visualizza il codice di errore HTTP. Il documento viene corretto e reinviato manualmente.</t>
+          <t>Errore notificato all'utente, con possibilità di correzione e reinvio tramite gestione applicativa e retry.</t>
         </is>
       </c>
       <c r="T189" s="62" t="inlineStr">

</xml_diff>